<commit_message>
n8n board refresh 2026-09-30T17:40:34Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-02 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.821</v>
+        <v>0.885</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>32.9</v>
+        <v>35.9</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>20.83</v>
+        <v>18.19</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.579</v>
+        <v>0.974</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.507</v>
+        <v>0.827</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04480999946594239</v>
+        <v>0.05302000045776367</v>
       </c>
     </row>
     <row r="6">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>3927000064</v>
+        <v>3824999936</v>
       </c>
     </row>
     <row r="33">
@@ -1199,7 +1199,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>428000000</v>
+        <v>459000000</v>
       </c>
     </row>
     <row r="34">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244316322.2275564</v>
+        <v>244506430.3463441</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>20.83</v>
+        <v>18.19</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>5089108992</v>
+        <v>4447571968</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>34.72</v>
+        <v>21.92</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.539999999999999</v>
+        <v>7.85</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>4644443648</v>
+        <v>3699812864</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>18.342262</v>
+        <v>16.222155</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>11.737</v>
+        <v>10.614</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.349</v>
+        <v>1.185</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>5963753472</v>
+        <v>6148728832</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>18.023605</v>
+        <v>17.260654</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>17.131</v>
+        <v>15.811</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.92</v>
+        <v>9.130000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>7366219264</v>
+        <v>6347076608</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>64.6755</v>
+        <v>42.38889</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>24.182</v>
+        <v>18.704</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>4.303</v>
+        <v>3.678</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4572046336</v>
+        <v>4446409728</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.637168</v>
+        <v>10.623494</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.428</v>
+        <v>10.252</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.887</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>13118161920</v>
+        <v>12129740800</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>46.838234</v>
+        <v>32.511883</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>25.543</v>
+        <v>21.116</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.474</v>
+        <v>3.093</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>7439963648</v>
+        <v>5066893312</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>80.517</v>
+        <v>65.583</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>7.977</v>
+        <v>5.346</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>7544854016</v>
+        <v>7710502400</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>24.187</v>
+        <v>21.959</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>4.233</v>
+        <v>3.978</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-01T17:40:22Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-01 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.885</v>
+        <v>0.883</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>35.9</v>
+        <v>36.64</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>18.19</v>
+        <v>18.67</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.974</v>
+        <v>0.963</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.827</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05302000045776367</v>
+        <v>0.05217999935150146</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244506430.3463441</v>
+        <v>244506408.9983931</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>18.19</v>
+        <v>18.67</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>4447571968</v>
+        <v>4564934656</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>21.92</v>
+        <v>22.49</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>7.85</v>
+        <v>7.84</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>0.5600000000000001</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>3699812864</v>
+        <v>3953287424</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>16.222155</v>
+        <v>17.333534</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.614</v>
+        <v>10.764</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.185</v>
+        <v>1.202</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>6148728832</v>
+        <v>5979264512</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>17.260654</v>
+        <v>16.768316</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.811</v>
+        <v>15.637</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.130000000000001</v>
+        <v>9.029999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6347076608</v>
+        <v>6514960896</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>42.38889</v>
+        <v>43.5101</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>18.704</v>
+        <v>18.62</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.678</v>
+        <v>3.661</v>
       </c>
     </row>
     <row r="9">
@@ -1616,13 +1616,13 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4446409728</v>
+        <v>4464058880</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.623494</v>
+        <v>10.665663</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.252</v>
+        <v>10.257</v>
       </c>
       <c r="F9" s="34" t="n">
         <v>0.895</v>
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12129740800</v>
+        <v>12445977600</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>32.511883</v>
+        <v>33.331215</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>21.116</v>
+        <v>20.81</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.093</v>
+        <v>3.048</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>5066893312</v>
+        <v>5109497856</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>65.583</v>
+        <v>65.85299999999999</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.346</v>
+        <v>5.368</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>7710502400</v>
+        <v>7780205568</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>21.959</v>
+        <v>21.732</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>3.978</v>
+        <v>3.937</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
n8n board refresh 2026-10-02T17:41:08Z
</commit_message>
<xml_diff>
--- a/app/reports/AMTM_research.xlsx
+++ b/app/reports/AMTM_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-01 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-02 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.883</v>
+        <v>0.887</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>36.64</v>
+        <v>36.12</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>18.67</v>
+        <v>17.975</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.963</v>
+        <v>1.009</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.834</v>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.05217999935150146</v>
+        <v>0.05276999950408936</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>244506408.9983931</v>
+        <v>244506418.9151599</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>18.67</v>
+        <v>17.975</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>4564934656</v>
+        <v>4395002880</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>22.49</v>
+        <v>21.66</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>7.84</v>
+        <v>7.93</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>0.5600000000000001</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>3953287424</v>
+        <v>3799905024</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>17.333534</v>
+        <v>16.661016</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>10.764</v>
+        <v>11.208</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>1.202</v>
+        <v>1.251</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>5979264512</v>
+        <v>6083767296</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>16.768316</v>
+        <v>17.061386</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>15.637</v>
+        <v>15.603</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>9.029999999999999</v>
+        <v>9.01</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>6514960896</v>
+        <v>6505885696</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>43.5101</v>
+        <v>43.449493</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>18.62</v>
+        <v>19.168</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.661</v>
+        <v>3.769</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>4464058880</v>
+        <v>4309626368</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>10.665663</v>
+        <v>10.296687</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>10.257</v>
+        <v>10.237</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.895</v>
+        <v>0.893</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>12445977600</v>
+        <v>12416998400</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>33.331215</v>
+        <v>33.281834</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>20.81</v>
+        <v>21.247</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.048</v>
+        <v>3.112</v>
       </c>
     </row>
     <row r="11">
@@ -1664,14 +1664,14 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>5109497856</v>
+        <v>5146929152</v>
       </c>
       <c r="D11" s="34" t="n"/>
       <c r="E11" s="34" t="n">
-        <v>65.85299999999999</v>
+        <v>66.655</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>5.368</v>
+        <v>5.433</v>
       </c>
     </row>
     <row r="12">
@@ -1686,14 +1686,14 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>7780205568</v>
+        <v>8214467584</v>
       </c>
       <c r="D12" s="34" t="n"/>
       <c r="E12" s="34" t="n">
-        <v>21.732</v>
+        <v>22.188</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>3.937</v>
+        <v>4.019</v>
       </c>
     </row>
     <row r="13">

</xml_diff>